<commit_message>
Add hero-video, parallax-collage blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 14
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-new-energy.report.xlsx
+++ b/tools/importer/reports/import-new-energy.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="41">
   <si>
     <t>_reportFile</t>
   </si>
@@ -76,31 +76,64 @@
     <t>MG Latest Luxury &amp; Electric Cars in India - Prices &amp; Models</t>
   </si>
   <si>
+    <t>jsw-nav.report.json</t>
+  </si>
+  <si>
+    <t>jsw-nav</t>
+  </si>
+  <si>
+    <t>nav</t>
+  </si>
+  <si>
+    <t>2026-10-09T05:25:33.686Z</t>
+  </si>
+  <si>
+    <t>JSW Motors navigation</t>
+  </si>
+  <si>
+    <t>http://localhost:3000/drafts/jsw-nav/source.html</t>
+  </si>
+  <si>
     <t>nav.report.json</t>
   </si>
   <si>
-    <t>nav</t>
-  </si>
-  <si>
     <t>2026-10-06T10:49:04.281Z</t>
   </si>
   <si>
     <t>new-energy.report.json</t>
   </si>
   <si>
-    <t>["hero-interactive"]</t>
+    <t>["hero-video"]</t>
   </si>
   <si>
     <t>new-energy</t>
   </si>
   <si>
-    <t>2026-10-08T19:27:02.871Z</t>
+    <t>2026-10-12T06:50:04.351Z</t>
   </si>
   <si>
     <t>New Energy | Built for Beyond</t>
   </si>
   <si>
     <t>http://localhost:3000/drafts/new-energy/source.html</t>
+  </si>
+  <si>
+    <t>sustainable-future.report.json</t>
+  </si>
+  <si>
+    <t>["parallax-collage"]</t>
+  </si>
+  <si>
+    <t>sustainable-future</t>
+  </si>
+  <si>
+    <t>2026-10-09T08:58:41.555Z</t>
+  </si>
+  <si>
+    <t>Driving India into a More Sustainable Future</t>
+  </si>
+  <si>
+    <t>http://localhost:3000/drafts/sustainable-future/source.html</t>
   </si>
 </sst>
 </file>
@@ -489,14 +522,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
     <col min="7" max="7" width="26" customWidth="1"/>
     <col min="8" max="9" width="50" customWidth="1"/>
   </cols>
@@ -598,52 +631,110 @@
       <c r="C4" t="s">
         <v>22</v>
       </c>
-      <c r="D4">
-        <v>6</v>
+      <c r="D4" t="s">
+        <v>10</v>
       </c>
       <c r="E4" t="s">
         <v>12</v>
       </c>
       <c r="F4" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="G4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I4" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="C5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D5" t="s">
-        <v>10</v>
+        <v>23</v>
+      </c>
+      <c r="D5">
+        <v>6</v>
       </c>
       <c r="E5" t="s">
         <v>12</v>
       </c>
       <c r="F5" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H5" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="I5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>29</v>
+      </c>
+      <c r="B6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" t="s">
+        <v>37</v>
+      </c>
+      <c r="G7" t="s">
+        <v>38</v>
+      </c>
+      <c r="H7" t="s">
+        <v>39</v>
+      </c>
+      <c r="I7" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add engine-showcase, hero-video blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 16
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-new-energy.report.xlsx
+++ b/tools/importer/reports/import-new-energy.report.xlsx
@@ -103,13 +103,13 @@
     <t>new-energy.report.json</t>
   </si>
   <si>
-    <t>["hero-video"]</t>
+    <t>["hero-video","engine-showcase"]</t>
   </si>
   <si>
     <t>new-energy</t>
   </si>
   <si>
-    <t>2026-10-12T06:50:04.351Z</t>
+    <t>2026-10-12T07:39:00.527Z</t>
   </si>
   <si>
     <t>New Energy | Built for Beyond</t>

</xml_diff>

<commit_message>
Add blog-carousel, parallax-collage blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 15
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-new-energy.report.xlsx
+++ b/tools/importer/reports/import-new-energy.report.xlsx
@@ -103,13 +103,13 @@
     <t>new-energy.report.json</t>
   </si>
   <si>
-    <t>["hero-video","engine-showcase","parallax-collage"]</t>
+    <t>["hero-video","engine-showcase","parallax-collage","blog-carousel"]</t>
   </si>
   <si>
     <t>new-energy</t>
   </si>
   <si>
-    <t>2026-10-12T19:12:41.374Z</t>
+    <t>2026-10-13T04:39:05.091Z</t>
   </si>
   <si>
     <t>New Energy | Built for Beyond</t>

</xml_diff>